<commit_message>
Drop unused Hotel.calling column; merge misspelled hotel area names
calling was always empty in practice, so remove it from the schema,
seed script, API select, and hotel detail view (migration applied
to production separately).

Also normalize duplicate/misspelled Hotel.area values that were
splitting the same location into multiple filter entries: Kiari and
"Ftehpur range kyari" -> Kyari, Mohan -> Mohaan, Choii/Madanpur
Chhoi/Khempur Chhoi -> Chhoi. Fixed in the source rate sheet too so
a future reseed doesn't reintroduce the split (live rows were
updated directly via a one-off script, already run).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/corbett-hotel-sheet.xlsx
+++ b/backend/data/corbett-hotel-sheet.xlsx
@@ -2818,7 +2818,7 @@
         <v>Green Retreat Resort</v>
       </c>
       <c r="B62" t="str">
-        <v>Madanpur Chhoi</v>
+        <v>Chhoi</v>
       </c>
       <c r="C62">
         <v>43</v>
@@ -4171,7 +4171,7 @@
         <v>Trinantara Resort &amp; Spa</v>
       </c>
       <c r="B98" t="str">
-        <v>Khempur Chhoi</v>
+        <v>Chhoi</v>
       </c>
       <c r="C98">
         <v>100</v>

</xml_diff>

<commit_message>
Clear contact-status notes typed into hotel rate/data fields
Follow-up notes like "Not Answering", "Message shared no response",
"Will arrange a call back", "Not able to connect", and "outside
vendor not allowed" had been typed into AP Plan Season Rate, Extra
Person Rate, Notes, and 2nd Contact Person instead of real data.

Fixed in the source rate sheet so a future reseed stays clean; the
live rows were cleared directly via a one-off script (already run).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/corbett-hotel-sheet.xlsx
+++ b/backend/data/corbett-hotel-sheet.xlsx
@@ -2151,9 +2151,6 @@
       <c r="K47" t="str">
         <v>9015242000</v>
       </c>
-      <c r="L47" t="str">
-        <v>Message shared no response</v>
-      </c>
       <c r="P47" t="str">
         <v>17</v>
       </c>
@@ -2533,9 +2530,6 @@
       <c r="H55" t="str">
         <v>info@clarissaresorts.com</v>
       </c>
-      <c r="L55" t="str">
-        <v>Message shared no response</v>
-      </c>
       <c r="S55" t="str">
         <v>Kashish</v>
       </c>
@@ -2715,9 +2709,6 @@
       <c r="H59" t="str">
         <v>sales@harmonyhotels.co.in</v>
       </c>
-      <c r="L59" t="str">
-        <v>Not Answering</v>
-      </c>
       <c r="P59" t="str">
         <v>120</v>
       </c>
@@ -2841,9 +2832,6 @@
       <c r="I62" t="str">
         <v>Anil</v>
       </c>
-      <c r="L62" t="str">
-        <v>Message shared no response</v>
-      </c>
       <c r="S62" t="str">
         <v>Kashish</v>
       </c>
@@ -2879,9 +2867,6 @@
       <c r="K63" t="str">
         <v>9520990494</v>
       </c>
-      <c r="L63" t="str">
-        <v>Message shared no response</v>
-      </c>
       <c r="P63" t="str">
         <v>144</v>
       </c>
@@ -2917,9 +2902,6 @@
       <c r="H64" t="str">
         <v>creekwoodresortkyari@gmail.com</v>
       </c>
-      <c r="L64" t="str">
-        <v>Message shared no response</v>
-      </c>
       <c r="S64" t="str">
         <v>Kashish</v>
       </c>
@@ -2996,9 +2978,6 @@
       <c r="H66" t="str">
         <v>crs@sterlingholidays.com</v>
       </c>
-      <c r="L66" t="str">
-        <v>Not Answering</v>
-      </c>
       <c r="S66" t="str">
         <v>Kashish</v>
       </c>
@@ -3019,9 +2998,6 @@
       <c r="H67" t="str">
         <v>sales@leroihotels.com</v>
       </c>
-      <c r="L67" t="str">
-        <v>Not Answering</v>
-      </c>
       <c r="S67" t="str">
         <v>Kashish</v>
       </c>
@@ -3253,9 +3229,6 @@
       <c r="D73" t="str">
         <v>https://www.makemytrip.com/hotels/address-of-bentocorbettwoodsresort-details_-jimcor_bettram_nagar._html_</v>
       </c>
-      <c r="L73" t="str">
-        <v>Not able to connect</v>
-      </c>
       <c r="S73" t="str">
         <v>Kashish</v>
       </c>
@@ -3352,9 +3325,6 @@
       <c r="H76" t="str">
         <v>reservations@aahmahospitality.com</v>
       </c>
-      <c r="N76" t="str">
-        <v>outside vendor not allowed</v>
-      </c>
       <c r="P76" t="str">
         <v>250-300</v>
       </c>
@@ -3378,9 +3348,6 @@
       <c r="H77" t="str">
         <v>sales@treffresort.com</v>
       </c>
-      <c r="L77" t="str">
-        <v>Will arrange a call back</v>
-      </c>
       <c r="S77" t="str">
         <v>Kashish</v>
       </c>
@@ -3424,9 +3391,6 @@
       <c r="H79" t="str">
         <v>info@tuskarsresort.com</v>
       </c>
-      <c r="L79" t="str">
-        <v>Will arrange a call back</v>
-      </c>
       <c r="P79" t="str">
         <v>60</v>
       </c>
@@ -3651,9 +3615,6 @@
       </c>
       <c r="H85" t="str">
         <v>info@sshubhhotels.com</v>
-      </c>
-      <c r="I85" t="str">
-        <v>Not able to connect</v>
       </c>
       <c r="S85" t="str">
         <v>Kashish</v>

</xml_diff>